<commit_message>
Update README.md with project description, prerequisites, and installation instructions
</commit_message>
<xml_diff>
--- a/IT23391222_Assignment 1 - Test cases.xlsx
+++ b/IT23391222_Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IT23391222\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A03E7A36-D738-44F8-B3ED-91D83DAEEF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B1652B-F440-4C88-B9AE-B7482593194D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="243">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -743,6 +743,12 @@
   </si>
   <si>
     <t>Rationale: includes date + file type + email</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>M</t>
   </si>
 </sst>
 </file>
@@ -1186,7 +1192,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>6</v>
+        <v>241</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>7</v>
@@ -1212,7 +1218,7 @@
         <v>10</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>10</v>
+        <v>241</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>11</v>
@@ -1238,7 +1244,7 @@
         <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>13</v>
+        <v>241</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>14</v>
@@ -1264,7 +1270,7 @@
         <v>16</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>16</v>
+        <v>241</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>17</v>
@@ -1290,7 +1296,7 @@
         <v>19</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>19</v>
+        <v>241</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>20</v>
@@ -1316,7 +1322,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>22</v>
+        <v>241</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>23</v>
@@ -1342,7 +1348,7 @@
         <v>25</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>25</v>
+        <v>242</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>26</v>
@@ -1368,7 +1374,7 @@
         <v>28</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>28</v>
+        <v>241</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>29</v>
@@ -1394,7 +1400,7 @@
         <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>31</v>
+        <v>241</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>32</v>
@@ -1420,7 +1426,7 @@
         <v>34</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>34</v>
+        <v>241</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>35</v>
@@ -1446,7 +1452,7 @@
         <v>37</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>37</v>
+        <v>241</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>38</v>
@@ -1472,7 +1478,7 @@
         <v>40</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>40</v>
+        <v>241</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>41</v>
@@ -1498,7 +1504,7 @@
         <v>43</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>43</v>
+        <v>241</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>44</v>
@@ -1524,7 +1530,7 @@
         <v>46</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>46</v>
+        <v>241</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>47</v>
@@ -1550,7 +1556,7 @@
         <v>50</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>50</v>
+        <v>241</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>51</v>
@@ -1576,7 +1582,7 @@
         <v>54</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>54</v>
+        <v>241</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>55</v>
@@ -1602,7 +1608,7 @@
         <v>57</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>57</v>
+        <v>241</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>58</v>
@@ -1628,7 +1634,7 @@
         <v>60</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>60</v>
+        <v>241</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>61</v>
@@ -1654,7 +1660,7 @@
         <v>63</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>63</v>
+        <v>242</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>64</v>
@@ -1758,7 +1764,7 @@
         <v>75</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>75</v>
+        <v>241</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>76</v>
@@ -1784,7 +1790,7 @@
         <v>78</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>78</v>
+        <v>241</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>79</v>
@@ -1810,7 +1816,7 @@
         <v>81</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>81</v>
+        <v>241</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>82</v>
@@ -1836,7 +1842,7 @@
         <v>84</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>84</v>
+        <v>241</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>85</v>
@@ -1862,7 +1868,7 @@
         <v>87</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>87</v>
+        <v>241</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>88</v>
@@ -1888,7 +1894,7 @@
         <v>90</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>90</v>
+        <v>241</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>91</v>
@@ -1914,7 +1920,7 @@
         <v>93</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>93</v>
+        <v>241</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>94</v>
@@ -1940,7 +1946,7 @@
         <v>96</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>96</v>
+        <v>241</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>97</v>
@@ -1966,7 +1972,7 @@
         <v>99</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>99</v>
+        <v>241</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>100</v>
@@ -1992,7 +1998,7 @@
         <v>102</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>102</v>
+        <v>241</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>103</v>
@@ -2018,7 +2024,7 @@
         <v>105</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>105</v>
+        <v>241</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>106</v>
@@ -2044,7 +2050,7 @@
         <v>109</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>109</v>
+        <v>241</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>110</v>
@@ -2070,7 +2076,7 @@
         <v>112</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>112</v>
+        <v>241</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>113</v>
@@ -2096,7 +2102,7 @@
         <v>115</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>115</v>
+        <v>241</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>116</v>
@@ -2122,7 +2128,7 @@
         <v>118</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>118</v>
+        <v>241</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>119</v>
@@ -2148,7 +2154,7 @@
         <v>121</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>121</v>
+        <v>241</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>122</v>
@@ -2174,7 +2180,7 @@
         <v>124</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>124</v>
+        <v>241</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>125</v>
@@ -2200,7 +2206,7 @@
         <v>127</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>127</v>
+        <v>241</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>128</v>
@@ -2226,7 +2232,7 @@
         <v>130</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>131</v>
@@ -2252,7 +2258,7 @@
         <v>133</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>133</v>
+        <v>241</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>134</v>
@@ -2278,7 +2284,7 @@
         <v>137</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>137</v>
+        <v>241</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>138</v>
@@ -2304,7 +2310,7 @@
         <v>140</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>140</v>
+        <v>241</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>141</v>
@@ -2330,7 +2336,7 @@
         <v>143</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>143</v>
+        <v>241</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>144</v>
@@ -2356,7 +2362,7 @@
         <v>146</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>146</v>
+        <v>241</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>147</v>
@@ -2382,7 +2388,7 @@
         <v>149</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>149</v>
+        <v>241</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>150</v>
@@ -2408,7 +2414,7 @@
         <v>152</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>152</v>
+        <v>241</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>153</v>
@@ -2434,7 +2440,7 @@
         <v>155</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>155</v>
+        <v>242</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>156</v>
@@ -2460,7 +2466,7 @@
         <v>158</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>158</v>
+        <v>242</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>159</v>

</xml_diff>